<commit_message>
Keep the Week 2 brief on the distance adjustment
The sample-size question pulled the student back to raw FG% right after
the assignment taught them to distrust it, and the adjusted rate's
interval is not the Week 2 formula. Question 4 now asks whether the
adjustment changes the answer about Aubrey. The margin-of-error note goes
with it, and the sheet description matches the trimmed worksheet.
</commit_message>
<xml_diff>
--- a/weeks/week02/data/hand-build-rates-and-intervals-worksheet.xlsx
+++ b/weeks/week02/data/hand-build-rates-and-intervals-worksheet.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T30"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -473,10 +473,6 @@
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,26 +549,6 @@
       <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Z score vs league</t>
-        </is>
-      </c>
-      <c r="Q1" s="2" t="inlineStr">
-        <is>
-          <t>Interval excludes league rate?</t>
-        </is>
-      </c>
-      <c r="R1" s="2" t="inlineStr">
-        <is>
-          <t>P(next two both made), multiplied</t>
-        </is>
-      </c>
-      <c r="S1" s="2" t="inlineStr">
-        <is>
-          <t>P(next two both made), BINOM.DIST</t>
-        </is>
-      </c>
-      <c r="T1" s="2" t="inlineStr">
-        <is>
-          <t>P(his makes or fewer, at the league rate)</t>
         </is>
       </c>
     </row>
@@ -612,10 +588,6 @@
         <v>0.8421999999999999</v>
       </c>
       <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1296,7 +1268,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Fill in every highlighted cell. Each one turns from yellow to green when the answer in it is right, so a sheet with any yellow left in it is not finished. The check allows for rounding, so a value you rounded to three decimals still turns green. Use cell references, not typed-in numbers, so the sheet still works if a row changes. The two P(next two both made) cells ask for the same probability twice, once by multiplying the rate by itself and once with BINOM.DIST. They should agree to every decimal, and if they do not, your BINOM.DIST arguments are in the wrong order.</t>
+          <t>Fill in every highlighted cell. Each one turns from yellow to green when the answer in it is right, so a sheet with any yellow left in it is not finished. The check allows for rounding, so a value you rounded to three decimals still turns green. Use cell references, not typed-in numbers, so the sheet still works if a row changes.</t>
         </is>
       </c>
     </row>
@@ -1339,26 +1311,6 @@
   <conditionalFormatting sqref="P2">
     <cfRule type="expression" priority="8" dxfId="0">
       <formula>AND(ISNUMBER(P2),ABS(P2-(((SUM($F$2:$F$28)/COUNT($D$2:$D$28))-$O$2)/(SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))))&lt;=MAX(0.02*ABS(((SUM($F$2:$F$28)/COUNT($D$2:$D$28))-$O$2)/(SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q2">
-    <cfRule type="expression" priority="9" dxfId="0">
-      <formula>AND(Q2&lt;&gt;"",EXACT(LOWER(TRIM(Q2)),LOWER(IF(OR((SUM($F$2:$F$28)/COUNT($D$2:$D$28))+(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))&lt;$O$2,(SUM($F$2:$F$28)/COUNT($D$2:$D$28))-(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))&gt;$O$2),"yes","no"))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R2">
-    <cfRule type="expression" priority="10" dxfId="0">
-      <formula>AND(ISNUMBER(R2),ABS(R2-((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(SUM($F$2:$F$28)/COUNT($D$2:$D$28))))&lt;=MAX(0.02*ABS((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(SUM($F$2:$F$28)/COUNT($D$2:$D$28))),0.005))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2">
-    <cfRule type="expression" priority="11" dxfId="0">
-      <formula>AND(ISNUMBER(S2),ABS(S2-((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(SUM($F$2:$F$28)/COUNT($D$2:$D$28))))&lt;=MAX(0.02*ABS((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(SUM($F$2:$F$28)/COUNT($D$2:$D$28))),0.005))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T2">
-    <cfRule type="expression" priority="12" dxfId="0">
-      <formula>AND(ISNUMBER(T2),ABS(T2-(_xlfn.BINOM.DIST(SUM($F$2:$F$28),COUNT($D$2:$D$28),$O$2,TRUE)))&lt;=MAX(0.02*ABS(_xlfn.BINOM.DIST(SUM($F$2:$F$28),COUNT($D$2:$D$28),$O$2,TRUE)),0.005))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>